<commit_message>
added gyro + magnetometer to BOM
</commit_message>
<xml_diff>
--- a/MM27/MM27_BillOfMaterials.xlsx
+++ b/MM27/MM27_BillOfMaterials.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tuprd-my.sharepoint.com/personal/tus21678_temple_edu/Documents/Classes/IEEE/Micromouse-2027/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\james\Documents\Github\micromouse-2027\MM27\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{8CE85860-FC5E-4D57-A2F2-879CDE2EC8F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F01AC708-05C2-4B20-967F-F7DB122CB74F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62813FAF-BC3B-473D-A790-67DA4E3CFAEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{919ED094-74B0-403E-90F8-720DCB4A05AB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{919ED094-74B0-403E-90F8-720DCB4A05AB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Parts</t>
   </si>
@@ -47,7 +47,28 @@
     <t xml:space="preserve">Microcontroller </t>
   </si>
   <si>
-    <t>https://www.digikey.com/en/products/detail/stmicroelectronics/NUCLEO-L432KC/6132763?gclid=aefe7fd242a218d3022f156c8eaae690&amp;gclsrc=3p.ds&amp;msclkid=aefe7fd242a218d3022f156c8eaae690</t>
+    <t>https://amazon.com/dp/B0GT32ZP55</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>acc + gyro</t>
+  </si>
+  <si>
+    <t>https://www.adafruit.com/product/4438</t>
+  </si>
+  <si>
+    <t>magnetometer</t>
+  </si>
+  <si>
+    <t>https://www.adafruit.com/product/4479</t>
+  </si>
+  <si>
+    <t>Cost</t>
+  </si>
+  <si>
+    <t>Quantity</t>
   </si>
 </sst>
 </file>
@@ -430,29 +451,72 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7324212C-B5B7-4243-BC11-99FB618AAEEC}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="91.6640625" customWidth="1"/>
+    <col min="2" max="2" width="91.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>2</v>
+      </c>
+      <c r="C2">
+        <v>7.99</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3">
+        <v>11.95</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4">
+        <v>9.9499999999999993</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{995D184B-3525-4F38-BF12-4283EB5BFCB8}"/>
+    <hyperlink ref="B2" r:id="rId1" tooltip="Original URL: https://amazon.com/dp/B0GT32ZP55. Click or tap if you trust this link." display="https://nam10.safelinks.protection.outlook.com/?url=https%3A%2F%2Famazon.com%2Fdp%2FB0GT32ZP55&amp;data=05%7C02%7Cjames.soley%40temple.edu%7C413a45dc57d64fa9f81508df24bde4c0%7C716e81efb52244738e3110bd02ccf6e5%7C0%7C0%7C639270070293192336%7CUnknown%7CTWFpbGZsb3d8eyJFbXB0eU1hcGkiOnRydWUsIlYiOiIwLjAuMDAwMCIsIlAiOiJXaW4zMiIsIkFOIjoiTWFpbCIsIldUIjoyfQ%3D%3D%7C60000%7C%7C%7C&amp;sdata=sO2zteh7pVfXOth3RCLsO%2FBYY75bLegm7ytU9%2B8EudA%3D&amp;reserved=0" xr:uid="{EAFA63BF-C6C7-405F-83AC-8C421B89B979}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
#GOATED We got the KiCad symbols and footprint ;)
</commit_message>
<xml_diff>
--- a/MM27/MM27_BillOfMaterials.xlsx
+++ b/MM27/MM27_BillOfMaterials.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\james\Documents\Github\micromouse-2027\MM27\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tuprd-my.sharepoint.com/personal/tus21678_temple_edu/Documents/GitHub/REALGit/micromouse-2027/MM27/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62813FAF-BC3B-473D-A790-67DA4E3CFAEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{62813FAF-BC3B-473D-A790-67DA4E3CFAEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{421A7147-B359-4444-9FEA-7F201B436C5D}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{919ED094-74B0-403E-90F8-720DCB4A05AB}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{919ED094-74B0-403E-90F8-720DCB4A05AB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -452,13 +452,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7324212C-B5B7-4243-BC11-99FB618AAEEC}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="91.6328125" customWidth="1"/>
+    <col min="2" max="2" width="91.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -472,7 +472,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -486,11 +486,11 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C3">
@@ -500,11 +500,11 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C4">
@@ -517,6 +517,8 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" tooltip="Original URL: https://amazon.com/dp/B0GT32ZP55. Click or tap if you trust this link." display="https://nam10.safelinks.protection.outlook.com/?url=https%3A%2F%2Famazon.com%2Fdp%2FB0GT32ZP55&amp;data=05%7C02%7Cjames.soley%40temple.edu%7C413a45dc57d64fa9f81508df24bde4c0%7C716e81efb52244738e3110bd02ccf6e5%7C0%7C0%7C639270070293192336%7CUnknown%7CTWFpbGZsb3d8eyJFbXB0eU1hcGkiOnRydWUsIlYiOiIwLjAuMDAwMCIsIlAiOiJXaW4zMiIsIkFOIjoiTWFpbCIsIldUIjoyfQ%3D%3D%7C60000%7C%7C%7C&amp;sdata=sO2zteh7pVfXOth3RCLsO%2FBYY75bLegm7ytU9%2B8EudA%3D&amp;reserved=0" xr:uid="{EAFA63BF-C6C7-405F-83AC-8C421B89B979}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{485F681F-E05D-4C63-9E46-AB0B9F8D2C78}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{A386CDAE-8078-4755-844E-BCBCAC261BBF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>